<commit_message>
Update Git_URL in Test Cases
</commit_message>
<xml_diff>
--- a/QA_Assignment_Gmail_Compose_TestCases_Incubyte.xlsx
+++ b/QA_Assignment_Gmail_Compose_TestCases_Incubyte.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ehaysau\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ericsson-my.sharepoint.com/personal/ayushi_a_shah_ericsson_com/Documents/Iteration-2_testCases/Documents/GitHub/Incubyte-QA-Assignment/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55847772-A18C-4F8C-8584-E49BE90D6B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D5233A5-DE6A-42DD-B967-3552FA15A896}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="215">
   <si>
     <t>TEST CASE DOCUMENT</t>
   </si>
@@ -853,12 +853,15 @@
   <si>
     <t>Git_URL</t>
   </si>
+  <si>
+    <t>https://github.com/Ayushi874/Incubyte-QA-Assignment</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -910,6 +913,14 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="17">
@@ -1043,10 +1054,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1126,15 +1138,18 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1145,7 +1160,8 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1460,8 +1476,8 @@
       <c r="B2" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="30"/>
     </row>
     <row r="3" spans="2:4" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
@@ -1519,17 +1535,17 @@
       <c r="B9" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>11</v>
+      <c r="C9" s="27" t="s">
+        <v>214</v>
       </c>
       <c r="D9" s="2"/>
     </row>
     <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B10" s="30" t="s">
+      <c r="B10" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="28"/>
-      <c r="D10" s="29"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="30"/>
     </row>
     <row r="11" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B11" s="3" t="s">
@@ -1560,6 +1576,9 @@
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C9" r:id="rId1" xr:uid="{7208393B-B950-4493-9416-8BC2160F0476}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1582,16 +1601,16 @@
     <row r="1" spans="1:9" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5"/>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-      <c r="I2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="30"/>
     </row>
     <row r="3" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
@@ -2271,13 +2290,13 @@
     <row r="1" spans="1:6" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5"/>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="32" t="s">
         <v>116</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="30"/>
     </row>
     <row r="3" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="17" t="s">
@@ -2624,12 +2643,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="32" t="s">
         <v>171</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="30"/>
     </row>
     <row r="4" spans="2:5" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="6" t="s">
@@ -2715,52 +2734,52 @@
       <c r="E10" s="26"/>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B13" s="34" t="s">
+      <c r="B13" s="35" t="s">
         <v>182</v>
       </c>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="29"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="30"/>
     </row>
     <row r="14" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="32" t="s">
+      <c r="B14" s="33" t="s">
         <v>183</v>
       </c>
-      <c r="C14" s="33"/>
-      <c r="D14" s="33"/>
-      <c r="E14" s="33"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="34"/>
+      <c r="E14" s="34"/>
     </row>
     <row r="15" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="32" t="s">
+      <c r="B15" s="33" t="s">
         <v>184</v>
       </c>
-      <c r="C15" s="33"/>
-      <c r="D15" s="33"/>
-      <c r="E15" s="33"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
     </row>
     <row r="16" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="32" t="s">
+      <c r="B16" s="33" t="s">
         <v>185</v>
       </c>
-      <c r="C16" s="33"/>
-      <c r="D16" s="33"/>
-      <c r="E16" s="33"/>
+      <c r="C16" s="34"/>
+      <c r="D16" s="34"/>
+      <c r="E16" s="34"/>
     </row>
     <row r="17" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="32" t="s">
+      <c r="B17" s="33" t="s">
         <v>186</v>
       </c>
-      <c r="C17" s="33"/>
-      <c r="D17" s="33"/>
-      <c r="E17" s="33"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="34"/>
     </row>
     <row r="18" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="32" t="s">
+      <c r="B18" s="33" t="s">
         <v>187</v>
       </c>
-      <c r="C18" s="33"/>
-      <c r="D18" s="33"/>
-      <c r="E18" s="33"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2774,4 +2793,10 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{92e84ceb-fbfd-47ab-be52-080c6b87953f}" enabled="0" method="" siteId="{92e84ceb-fbfd-47ab-be52-080c6b87953f}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>